<commit_message>
tweaks and rewrite of kgstore to make it more rational
</commit_message>
<xml_diff>
--- a/src/kgraph/ontologies/kgmeta_vocab.xlsx
+++ b/src/kgraph/ontologies/kgmeta_vocab.xlsx
@@ -127,7 +127,7 @@
     <t xml:space="preserve">Object, Individual</t>
   </si>
   <si>
-    <t xml:space="preserve">An Entity is an individual node within a knowledge graph. It will typically be assigned a URI that identifies it.</t>
+    <t xml:space="preserve">An Entity is an individual node within a knowledge graph. It will represent a specific instance of something in the domain of discourse and is typically assigned a URI that identifies it uniquely.</t>
   </si>
   <si>
     <t xml:space="preserve">Literal</t>
@@ -347,7 +347,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -388,11 +388,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -455,7 +450,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -493,10 +488,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1202,10 +1193,10 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="11" t="s">
+      <c r="A21" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="8" t="s">
@@ -1229,10 +1220,10 @@
       <c r="S21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="11" t="s">
+      <c r="A22" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="8" t="s">
@@ -1253,10 +1244,10 @@
       <c r="S22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" s="11" t="s">
+      <c r="A23" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C23" s="8" t="s">
@@ -1277,10 +1268,10 @@
       <c r="S23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="11" t="s">
+      <c r="A24" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="8" t="s">
@@ -1301,10 +1292,10 @@
       <c r="S24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" s="11" t="s">
+      <c r="A25" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -1328,10 +1319,10 @@
       <c r="S25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" s="11" t="s">
+      <c r="A26" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C26" s="8" t="s">
@@ -1357,10 +1348,10 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" s="11" t="s">
+      <c r="A27" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="8" t="s">
@@ -1381,10 +1372,10 @@
       <c r="S27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" s="11" t="s">
+      <c r="A28" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C28" s="8" t="s">
@@ -1402,10 +1393,10 @@
       <c r="S28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" s="11" t="s">
+      <c r="A29" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C29" s="8" t="s">

</xml_diff>